<commit_message>
feat(fixtures): actualizar catálogo golden y corpus comercial 2027.
</commit_message>
<xml_diff>
--- a/fixtures/catalog/sample-catalog.xlsx
+++ b/fixtures/catalog/sample-catalog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="93">
   <si>
     <t>sku</t>
   </si>
@@ -40,43 +40,43 @@
     <t>estado</t>
   </si>
   <si>
-    <t>BODA-J1-ESENCIAL</t>
-  </si>
-  <si>
-    <t>Boda Esencial Jardín 1</t>
+    <t>EVT-J1-TC</t>
+  </si>
+  <si>
+    <t>Paquete Estándar</t>
   </si>
   <si>
     <t>boda</t>
   </si>
   <si>
-    <t>jardin-1</t>
-  </si>
-  <si>
-    <t>Paquete base para bodas en Jardín 1</t>
+    <t>tequesquitengo</t>
+  </si>
+  <si>
+    <t>Paquete Bodas 2027 en Tres Cielos Tequesquitengo: evento de tres días (viernes cortesía, sábado gran evento, domingo parrillada). Tarifas por tramo de invitados; no incluye IVA ni tramitología.</t>
   </si>
   <si>
     <t>publicado</t>
   </si>
   <si>
-    <t>BODA-J1-PREMIUM</t>
-  </si>
-  <si>
-    <t>Boda Premium Jardín 1</t>
-  </si>
-  <si>
-    <t>Paquete premium con catering ampliado</t>
-  </si>
-  <si>
-    <t>XV-J1-CLASICO</t>
-  </si>
-  <si>
-    <t>XV Clásico Jardín 1</t>
-  </si>
-  <si>
-    <t>xv</t>
-  </si>
-  <si>
-    <t>Celebración de XV años</t>
+    <t>EVT-J1-PREMIUM</t>
+  </si>
+  <si>
+    <t>Upgrade Premium</t>
+  </si>
+  <si>
+    <t>Todo el Paquete Estándar más table styling, barra de servicio/DJ booth, barra libre nacional, sillas premium, plafón de diseño y menú 100% res.</t>
+  </si>
+  <si>
+    <t>RENTA-J1</t>
+  </si>
+  <si>
+    <t>Solo renta</t>
+  </si>
+  <si>
+    <t>multi</t>
+  </si>
+  <si>
+    <t>Locación 11 h con carpa de cocina, limpieza, suite y valet. No incluye planta de luz ni banquete. Sin tarifa publicada en la ficha Bodas 2027.</t>
   </si>
   <si>
     <t>moneda</t>
@@ -106,19 +106,43 @@
     <t>MXN</t>
   </si>
   <si>
-    <t>evento</t>
-  </si>
-  <si>
-    <t>2026-01-01</t>
-  </si>
-  <si>
-    <t>2026-12-31</t>
-  </si>
-  <si>
-    <t>Anticipo 30%</t>
-  </si>
-  <si>
-    <t>Anticipo 40%</t>
+    <t>persona</t>
+  </si>
+  <si>
+    <t>2027-01-01</t>
+  </si>
+  <si>
+    <t>2027-12-31</t>
+  </si>
+  <si>
+    <t>Paquete Estándar 2027. 100 invitados. No incluye IVA ni tramitología.</t>
+  </si>
+  <si>
+    <t>Paquete Estándar 2027. 150 invitados. No incluye IVA ni tramitología.</t>
+  </si>
+  <si>
+    <t>Paquete Estándar 2027. 200 invitados. No incluye IVA ni tramitología.</t>
+  </si>
+  <si>
+    <t>Paquete Estándar 2027. 250 invitados. No incluye IVA ni tramitología.</t>
+  </si>
+  <si>
+    <t>Paquete Estándar 2027. 300 invitados. No incluye IVA ni tramitología.</t>
+  </si>
+  <si>
+    <t>Upgrade Premium 2027. 100 invitados. No incluye IVA ni tramitología.</t>
+  </si>
+  <si>
+    <t>Upgrade Premium 2027. 150 invitados. No incluye IVA ni tramitología.</t>
+  </si>
+  <si>
+    <t>Upgrade Premium 2027. 200 invitados. No incluye IVA ni tramitología.</t>
+  </si>
+  <si>
+    <t>Upgrade Premium 2027. 250 invitados. No incluye IVA ni tramitología.</t>
+  </si>
+  <si>
+    <t>Upgrade Premium 2027. 300 invitados. No incluye IVA ni tramitología.</t>
   </si>
   <si>
     <t>categoria</t>
@@ -130,40 +154,85 @@
     <t>obligatoria</t>
   </si>
   <si>
+    <t>otro</t>
+  </si>
+  <si>
+    <t>Evento de tres días: viernes cortesía, sábado gran evento y domingo parrillada</t>
+  </si>
+  <si>
+    <t>dias</t>
+  </si>
+  <si>
+    <t>Renta del jardín por 11 horas (estacionamiento, baños, áreas comunes)</t>
+  </si>
+  <si>
+    <t>horas</t>
+  </si>
+  <si>
+    <t>Suite nupcial queen size, dos noches</t>
+  </si>
+  <si>
+    <t>noches</t>
+  </si>
+  <si>
+    <t>personal</t>
+  </si>
+  <si>
+    <t>Valet para el 100% de los invitados</t>
+  </si>
+  <si>
+    <t>porciento_invitados</t>
+  </si>
+  <si>
+    <t>Capilla techada y consagrada</t>
+  </si>
+  <si>
+    <t>sillas</t>
+  </si>
+  <si>
     <t>catering</t>
   </si>
   <si>
-    <t>Menú tres tiempos</t>
+    <t>Banquete 3 tiempos (50% res y 50% pollo o cerdo)</t>
+  </si>
+  <si>
+    <t>tiempos</t>
+  </si>
+  <si>
+    <t>audio</t>
+  </si>
+  <si>
+    <t>DJ por todo el evento</t>
   </si>
   <si>
     <t>servicio</t>
   </si>
   <si>
+    <t>In House Planner (coordinación antes y durante el evento)</t>
+  </si>
+  <si>
+    <t>Banquete 3 tiempos base 100% res</t>
+  </si>
+  <si>
+    <t>Barra libre nacional (tequila tradicional, ron Matusalem, vodka Stolichnaya, whisky etiqueta roja)</t>
+  </si>
+  <si>
     <t>mobiliario</t>
   </si>
   <si>
-    <t>Mobiliario básico</t>
-  </si>
-  <si>
-    <t>paquete</t>
-  </si>
-  <si>
-    <t>Menú premium + barra libre 4h</t>
-  </si>
-  <si>
-    <t>audio</t>
-  </si>
-  <si>
-    <t>Audio profesional</t>
-  </si>
-  <si>
-    <t>set</t>
-  </si>
-  <si>
-    <t>decoracion</t>
-  </si>
-  <si>
-    <t>Decoración temática</t>
+    <t>Table styling (copas, plato base y plaqué de color)</t>
+  </si>
+  <si>
+    <t>Sillas premium y plafón de diseño</t>
+  </si>
+  <si>
+    <t>DJ por todo el evento y upgrade de barra de servicio / DJ booth</t>
+  </si>
+  <si>
+    <t>Renta del jardín por 11 horas (estacionamiento, baños, áreas comunes, carpa de cocina)</t>
+  </si>
+  <si>
+    <t>Valet y personal de limpieza. No incluye planta de luz ni banquete</t>
   </si>
   <si>
     <t>tipo</t>
@@ -178,19 +247,52 @@
     <t>anticipo_minimo</t>
   </si>
   <si>
-    <t>{"anticipo_pct":30}</t>
-  </si>
-  <si>
-    <t>Se requiere anticipo del 30% para apartar la fecha.</t>
-  </si>
-  <si>
-    <t>solo_fin_semana</t>
-  </si>
-  <si>
-    <t>{}</t>
-  </si>
-  <si>
-    <t>El paquete Premium aplica solo fines de semana.</t>
+    <t>{"anticipo_pct":20,"momento":"firma_contrato"}</t>
+  </si>
+  <si>
+    <t>A la firma del contrato se requiere anticipo del 20%.</t>
+  </si>
+  <si>
+    <t>horario</t>
+  </si>
+  <si>
+    <t>{"horas_locacion_jardin":11}</t>
+  </si>
+  <si>
+    <t>El jardín se renta 11 horas el sábado. Meseros y mezcladores cubren 10 horas de servicio.</t>
+  </si>
+  <si>
+    <t>{"iva_incluido":false,"tramitologia_incluida":false}</t>
+  </si>
+  <si>
+    <t>Los precios no incluyen IVA ni tramitología.</t>
+  </si>
+  <si>
+    <t>{"liquidar_dias_antes_evento":30}</t>
+  </si>
+  <si>
+    <t>El saldo se liquida 30 días antes del evento.</t>
+  </si>
+  <si>
+    <t>{"temporada_baja":"jun-sep","descuento_desde":30000}</t>
+  </si>
+  <si>
+    <t>De junio a septiembre hay temporada baja con descuentos desde MXN 30,000. El monto exacto lo confirma un asesor.</t>
+  </si>
+  <si>
+    <t>{"aforo_tramos_publicados":[100,150,200,250,300],"interpolar":false}</t>
+  </si>
+  <si>
+    <t>Las tarifas publicadas son por tramos de 100, 150, 200, 250 y 300 invitados. Otros tamaños los confirma un asesor.</t>
+  </si>
+  <si>
+    <t>A la firma del contrato se requiere anticipo del 20%. Solo renta no tiene tarifa publicada en la ficha Bodas 2027; un asesor cotiza.</t>
+  </si>
+  <si>
+    <t>{"incluye_planta_luz":false}</t>
+  </si>
+  <si>
+    <t>Solo renta no incluye planta de luz ni banquete.</t>
   </si>
 </sst>
 </file>
@@ -610,10 +712,10 @@
         <v>11</v>
       </c>
       <c r="E2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F2">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="G2" t="s">
         <v>12</v>
@@ -639,7 +741,7 @@
         <v>100</v>
       </c>
       <c r="F3">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="G3" t="s">
         <v>16</v>
@@ -662,10 +764,10 @@
         <v>11</v>
       </c>
       <c r="E4">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>120</v>
+        <v>999</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
@@ -682,7 +784,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -722,7 +824,13 @@
         <v>29</v>
       </c>
       <c r="C2">
-        <v>85000</v>
+        <v>2980</v>
+      </c>
+      <c r="D2">
+        <v>100</v>
+      </c>
+      <c r="E2">
+        <v>100</v>
       </c>
       <c r="F2" t="s">
         <v>30</v>
@@ -739,13 +847,19 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>29</v>
       </c>
       <c r="C3">
-        <v>145000</v>
+        <v>2550</v>
+      </c>
+      <c r="D3">
+        <v>150</v>
+      </c>
+      <c r="E3">
+        <v>150</v>
       </c>
       <c r="F3" t="s">
         <v>30</v>
@@ -762,13 +876,19 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
         <v>29</v>
       </c>
       <c r="C4">
-        <v>62000</v>
+        <v>2200</v>
+      </c>
+      <c r="D4">
+        <v>200</v>
+      </c>
+      <c r="E4">
+        <v>200</v>
       </c>
       <c r="F4" t="s">
         <v>30</v>
@@ -778,6 +898,212 @@
       </c>
       <c r="H4" t="s">
         <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5">
+        <v>2000</v>
+      </c>
+      <c r="D5">
+        <v>250</v>
+      </c>
+      <c r="E5">
+        <v>250</v>
+      </c>
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6">
+        <v>1800</v>
+      </c>
+      <c r="D6">
+        <v>300</v>
+      </c>
+      <c r="E6">
+        <v>300</v>
+      </c>
+      <c r="F6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7">
+        <v>3590</v>
+      </c>
+      <c r="D7">
+        <v>100</v>
+      </c>
+      <c r="E7">
+        <v>100</v>
+      </c>
+      <c r="F7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8">
+        <v>3100</v>
+      </c>
+      <c r="D8">
+        <v>150</v>
+      </c>
+      <c r="E8">
+        <v>150</v>
+      </c>
+      <c r="F8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9">
+        <v>2710</v>
+      </c>
+      <c r="D9">
+        <v>200</v>
+      </c>
+      <c r="E9">
+        <v>200</v>
+      </c>
+      <c r="F9" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10">
+        <v>2450</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10">
+        <v>250</v>
+      </c>
+      <c r="F10" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H10" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11">
+        <v>2250</v>
+      </c>
+      <c r="D11">
+        <v>300</v>
+      </c>
+      <c r="E11">
+        <v>300</v>
+      </c>
+      <c r="F11" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -788,7 +1114,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -796,19 +1122,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="E1" t="s">
         <v>25</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -816,16 +1142,16 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -836,16 +1162,16 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -853,19 +1179,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -873,19 +1199,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="E5" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -893,22 +1219,302 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6">
+        <v>50</v>
+      </c>
+      <c r="E6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12">
+        <v>2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>63</v>
+      </c>
+      <c r="F14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15" t="s">
+        <v>63</v>
+      </c>
+      <c r="F15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>63</v>
+      </c>
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="s">
+        <v>63</v>
+      </c>
+      <c r="F17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>17</v>
       </c>
-      <c r="B6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F6" t="b">
-        <v>0</v>
+      <c r="B18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" t="s">
+        <v>72</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" t="s">
+        <v>63</v>
+      </c>
+      <c r="F20" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -919,7 +1525,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -927,13 +1533,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="C1" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="D1" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -941,13 +1547,13 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -955,13 +1561,181 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="D3" t="s">
-        <v>58</v>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" t="s">
+        <v>88</v>
+      </c>
+      <c r="D12" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" t="s">
+        <v>91</v>
+      </c>
+      <c r="D15" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>